<commit_message>
layout fixes; more named reefs; logos; other-living-benthos cap; dhw intervals
</commit_message>
<xml_diff>
--- a/www/Baseline_Cover_EXAMPLE.xlsx
+++ b/www/Baseline_Cover_EXAMPLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6203238-3524-411C-9A86-AB91011EA1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C85439B1-3D57-46A6-83EC-6019CFC36D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2543" yWindow="2543" windowWidth="21600" windowHeight="11332" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="137">
   <si>
     <t>Coral Cover Data Input README:</t>
   </si>
@@ -473,16 +473,61 @@
   <si>
     <t>john.morris@noaa.gov</t>
   </si>
+  <si>
+    <t>REQUIRED Other living benthos</t>
+  </si>
+  <si>
+    <t>Eastern Dry Rocks 10</t>
+  </si>
+  <si>
+    <t>LK_1354_Y2017</t>
+  </si>
+  <si>
+    <t>LK_1333_Y2015</t>
+  </si>
+  <si>
+    <t>LK_1434_Y2015</t>
+  </si>
+  <si>
+    <t>UK_1584_Y2015</t>
+  </si>
+  <si>
+    <t>UK_1271_Y2025</t>
+  </si>
+  <si>
+    <t>UK_1211_Y2015</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -531,6 +576,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -552,19 +602,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -596,9 +649,9 @@
       <sheetName val="Metadata"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
       <sheetData sheetId="3">
         <row r="2">
           <cell r="A2" t="str">
@@ -1920,7 +1973,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K1000"/>
+  <dimension ref="A1:K1008"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22.1328125" customWidth="1"/>
@@ -1928,7 +1981,7 @@
     <col min="3" max="3" width="9.1328125" customWidth="1"/>
     <col min="4" max="4" width="6.86328125" customWidth="1"/>
     <col min="5" max="5" width="13.1328125" customWidth="1"/>
-    <col min="6" max="6" width="9.3984375" customWidth="1"/>
+    <col min="6" max="6" width="21.19921875" customWidth="1"/>
     <col min="7" max="7" width="14.265625" customWidth="1"/>
     <col min="8" max="8" width="12.73046875" customWidth="1"/>
     <col min="9" max="9" width="11.59765625" customWidth="1"/>
@@ -2079,10 +2132,10 @@
     </row>
     <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B5" s="2">
-        <v>5</v>
+        <v>129</v>
+      </c>
+      <c r="B5" s="11">
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>31</v>
@@ -2090,10 +2143,10 @@
       <c r="D5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="11" t="s">
         <v>36</v>
       </c>
       <c r="G5" s="5">
@@ -2114,10 +2167,10 @@
     </row>
     <row r="6" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="B6" s="2">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>31</v>
@@ -2149,10 +2202,10 @@
     </row>
     <row r="7" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="B7" s="2">
-        <v>7.7</v>
+        <v>0.1</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>31</v>
@@ -2161,16 +2214,16 @@
         <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>36</v>
       </c>
       <c r="G7" s="5">
-        <v>24.45889</v>
+        <v>24.459129999999998</v>
       </c>
       <c r="H7" s="5">
-        <v>-81.846019999999996</v>
+        <v>-81.845830000000007</v>
       </c>
       <c r="I7" s="2">
         <v>100</v>
@@ -2184,10 +2237,10 @@
     </row>
     <row r="8" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>126</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2">
-        <v>2</v>
+        <v>7.7</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>31</v>
@@ -2198,8 +2251,8 @@
       <c r="E8" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>36</v>
+      <c r="F8" s="10" t="s">
+        <v>130</v>
       </c>
       <c r="G8" s="5">
         <v>24.45889</v>
@@ -2219,7 +2272,7 @@
     </row>
     <row r="9" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -2228,71 +2281,71 @@
         <v>31</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G9" s="2">
-        <v>24.616584899999999</v>
-      </c>
-      <c r="H9" s="2">
-        <v>-81.390728699999997</v>
+        <v>85</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="G9" s="5">
+        <v>24.45889</v>
+      </c>
+      <c r="H9" s="5">
+        <v>-81.846019999999996</v>
       </c>
       <c r="I9" s="2">
         <v>100</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>128</v>
+      <c r="J9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="2">
-        <v>6</v>
+        <v>129</v>
+      </c>
+      <c r="B10" s="10">
+        <v>0</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>106</v>
+        <v>33</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G10" s="2">
-        <v>24.616584899999999</v>
-      </c>
-      <c r="H10" s="2">
-        <v>-81.390728699999997</v>
+        <v>130</v>
+      </c>
+      <c r="G10" s="5">
+        <v>24.45889</v>
+      </c>
+      <c r="H10" s="5">
+        <v>-81.846019999999996</v>
       </c>
       <c r="I10" s="2">
         <v>100</v>
       </c>
-      <c r="J10" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>128</v>
+      <c r="J10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="B11" s="2">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>31</v>
@@ -2324,28 +2377,28 @@
     </row>
     <row r="12" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B12" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="G12" s="2">
-        <v>25.036133329999998</v>
+        <v>24.616584899999999</v>
       </c>
       <c r="H12" s="2">
-        <v>-80.346000000000004</v>
+        <v>-81.390728699999997</v>
       </c>
       <c r="I12" s="2">
         <v>100</v>
@@ -2359,28 +2412,28 @@
     </row>
     <row r="13" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="B13" s="2">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="G13" s="2">
-        <v>25.036133329999998</v>
+        <v>24.616584899999999</v>
       </c>
       <c r="H13" s="2">
-        <v>-80.346000000000004</v>
+        <v>-81.390728699999997</v>
       </c>
       <c r="I13" s="2">
         <v>100</v>
@@ -2394,28 +2447,28 @@
     </row>
     <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" s="2">
-        <v>1</v>
+        <v>129</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="G14" s="2">
-        <v>25.036133329999998</v>
+        <v>24.616584899999999</v>
       </c>
       <c r="H14" s="2">
-        <v>-80.346000000000004</v>
+        <v>-81.390728699999997</v>
       </c>
       <c r="I14" s="2">
         <v>100</v>
@@ -2429,10 +2482,10 @@
     </row>
     <row r="15" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B15" s="2">
-        <v>6.5</v>
+        <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>110</v>
@@ -2464,10 +2517,10 @@
     </row>
     <row r="16" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>126</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>110</v>
@@ -2499,28 +2552,28 @@
     </row>
     <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="B17" s="2">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="G17" s="2">
-        <v>24.456499999999998</v>
+        <v>25.036133329999998</v>
       </c>
       <c r="H17" s="2">
-        <v>-81.868700000000004</v>
+        <v>-80.346000000000004</v>
       </c>
       <c r="I17" s="2">
         <v>100</v>
@@ -2534,28 +2587,28 @@
     </row>
     <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="B18" s="2">
-        <v>1.5</v>
+        <v>6.5</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="G18" s="2">
-        <v>24.456499999999998</v>
+        <v>25.036133329999998</v>
       </c>
       <c r="H18" s="2">
-        <v>-81.868700000000004</v>
+        <v>-80.346000000000004</v>
       </c>
       <c r="I18" s="2">
         <v>100</v>
@@ -2569,28 +2622,28 @@
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>126</v>
       </c>
       <c r="B19" s="2">
-        <v>7.5</v>
+        <v>19</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="G19" s="2">
-        <v>24.456499999999998</v>
+        <v>25.036133329999998</v>
       </c>
       <c r="H19" s="2">
-        <v>-81.868700000000004</v>
+        <v>-80.346000000000004</v>
       </c>
       <c r="I19" s="2">
         <v>100</v>
@@ -2604,28 +2657,28 @@
     </row>
     <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B20" s="2">
-        <v>15.5</v>
+        <v>129</v>
+      </c>
+      <c r="B20" s="10">
+        <v>3</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="G20" s="2">
-        <v>24.456499999999998</v>
+        <v>25.036133329999998</v>
       </c>
       <c r="H20" s="2">
-        <v>-81.868700000000004</v>
+        <v>-80.346000000000004</v>
       </c>
       <c r="I20" s="2">
         <v>100</v>
@@ -2639,28 +2692,28 @@
     </row>
     <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B21" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="G21" s="2">
-        <v>24.885100000000001</v>
+        <v>24.456499999999998</v>
       </c>
       <c r="H21" s="2">
-        <v>-80.551439999999999</v>
+        <v>-81.868700000000004</v>
       </c>
       <c r="I21" s="2">
         <v>100</v>
@@ -2674,28 +2727,28 @@
     </row>
     <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="B22" s="2">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="G22" s="2">
-        <v>24.885100000000001</v>
+        <v>24.456499999999998</v>
       </c>
       <c r="H22" s="2">
-        <v>-80.551439999999999</v>
+        <v>-81.868700000000004</v>
       </c>
       <c r="I22" s="2">
         <v>100</v>
@@ -2709,28 +2762,28 @@
     </row>
     <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="B23" s="2">
-        <v>2</v>
+        <v>7.5</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="G23" s="2">
-        <v>24.885100000000001</v>
+        <v>24.456499999999998</v>
       </c>
       <c r="H23" s="2">
-        <v>-80.551439999999999</v>
+        <v>-81.868700000000004</v>
       </c>
       <c r="I23" s="2">
         <v>100</v>
@@ -2744,28 +2797,28 @@
     </row>
     <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>28</v>
+        <v>126</v>
       </c>
       <c r="B24" s="2">
-        <v>6</v>
+        <v>15.5</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="G24" s="2">
-        <v>24.885100000000001</v>
+        <v>24.456499999999998</v>
       </c>
       <c r="H24" s="2">
-        <v>-80.551439999999999</v>
+        <v>-81.868700000000004</v>
       </c>
       <c r="I24" s="2">
         <v>100</v>
@@ -2779,10 +2832,10 @@
     </row>
     <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>126</v>
+        <v>15</v>
       </c>
       <c r="B25" s="2">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>110</v>
@@ -2814,10 +2867,10 @@
     </row>
     <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B26" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>110</v>
@@ -2826,16 +2879,16 @@
         <v>33</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G26" s="2">
-        <v>24.910219999999999</v>
+        <v>24.885100000000001</v>
       </c>
       <c r="H26" s="2">
-        <v>-80.506519999999995</v>
+        <v>-80.551439999999999</v>
       </c>
       <c r="I26" s="2">
         <v>100</v>
@@ -2849,10 +2902,10 @@
     </row>
     <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="B27" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>110</v>
@@ -2861,16 +2914,16 @@
         <v>33</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G27" s="2">
-        <v>24.910219999999999</v>
+        <v>24.885100000000001</v>
       </c>
       <c r="H27" s="2">
-        <v>-80.506519999999995</v>
+        <v>-80.551439999999999</v>
       </c>
       <c r="I27" s="2">
         <v>100</v>
@@ -2884,10 +2937,10 @@
     </row>
     <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="B28" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>110</v>
@@ -2896,16 +2949,16 @@
         <v>33</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G28" s="2">
-        <v>24.910219999999999</v>
+        <v>24.885100000000001</v>
       </c>
       <c r="H28" s="2">
-        <v>-80.506519999999995</v>
+        <v>-80.551439999999999</v>
       </c>
       <c r="I28" s="2">
         <v>100</v>
@@ -2919,10 +2972,10 @@
     </row>
     <row r="29" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>27</v>
+        <v>126</v>
       </c>
       <c r="B29" s="2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>110</v>
@@ -2931,16 +2984,16 @@
         <v>33</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G29" s="2">
-        <v>24.910219999999999</v>
+        <v>24.885100000000001</v>
       </c>
       <c r="H29" s="2">
-        <v>-80.506519999999995</v>
+        <v>-80.551439999999999</v>
       </c>
       <c r="I29" s="2">
         <v>100</v>
@@ -2954,10 +3007,10 @@
     </row>
     <row r="30" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B30" s="2">
-        <v>1</v>
+        <v>129</v>
+      </c>
+      <c r="B30" s="10">
+        <v>1.5</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>110</v>
@@ -2966,16 +3019,16 @@
         <v>33</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="G30" s="2">
-        <v>24.910219999999999</v>
+        <v>24.885100000000001</v>
       </c>
       <c r="H30" s="2">
-        <v>-80.506519999999995</v>
+        <v>-80.551439999999999</v>
       </c>
       <c r="I30" s="2">
         <v>100</v>
@@ -2989,10 +3042,10 @@
     </row>
     <row r="31" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>98</v>
+        <v>15</v>
       </c>
       <c r="B31" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>110</v>
@@ -3024,10 +3077,10 @@
     </row>
     <row r="32" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B32" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>110</v>
@@ -3059,10 +3112,10 @@
     </row>
     <row r="33" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="B33" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>110</v>
@@ -3094,10 +3147,10 @@
     </row>
     <row r="34" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>126</v>
+        <v>27</v>
       </c>
       <c r="B34" s="2">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>110</v>
@@ -3129,28 +3182,28 @@
     </row>
     <row r="35" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="B35" s="2">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G35" s="2">
-        <v>25.215733329999999</v>
+        <v>24.910219999999999</v>
       </c>
       <c r="H35" s="2">
-        <v>-80.228566670000006</v>
+        <v>-80.506519999999995</v>
       </c>
       <c r="I35" s="2">
         <v>100</v>
@@ -3164,28 +3217,28 @@
     </row>
     <row r="36" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B36" s="2">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G36" s="2">
-        <v>25.215733329999999</v>
+        <v>24.910219999999999</v>
       </c>
       <c r="H36" s="2">
-        <v>-80.228566670000006</v>
+        <v>-80.506519999999995</v>
       </c>
       <c r="I36" s="2">
         <v>100</v>
@@ -3199,28 +3252,28 @@
     </row>
     <row r="37" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="B37" s="2">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G37" s="2">
-        <v>25.215733329999999</v>
+        <v>24.910219999999999</v>
       </c>
       <c r="H37" s="2">
-        <v>-80.228566670000006</v>
+        <v>-80.506519999999995</v>
       </c>
       <c r="I37" s="2">
         <v>100</v>
@@ -3237,25 +3290,25 @@
         <v>28</v>
       </c>
       <c r="B38" s="2">
-        <v>8.5</v>
+        <v>0</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G38" s="2">
-        <v>25.215733329999999</v>
+        <v>24.910219999999999</v>
       </c>
       <c r="H38" s="2">
-        <v>-80.228566670000006</v>
+        <v>-80.506519999999995</v>
       </c>
       <c r="I38" s="2">
         <v>100</v>
@@ -3272,25 +3325,25 @@
         <v>126</v>
       </c>
       <c r="B39" s="2">
-        <v>22.5</v>
+        <v>35</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G39" s="2">
-        <v>25.215733329999999</v>
+        <v>24.910219999999999</v>
       </c>
       <c r="H39" s="2">
-        <v>-80.228566670000006</v>
+        <v>-80.506519999999995</v>
       </c>
       <c r="I39" s="2">
         <v>100</v>
@@ -3304,10 +3357,10 @@
     </row>
     <row r="40" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B40" s="2">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>110</v>
@@ -3316,16 +3369,16 @@
         <v>117</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G40" s="2">
-        <v>24.934650000000001</v>
+        <v>25.215733329999999</v>
       </c>
       <c r="H40" s="2">
-        <v>-80.548766670000006</v>
+        <v>-80.228566670000006</v>
       </c>
       <c r="I40" s="2">
         <v>100</v>
@@ -3339,10 +3392,10 @@
     </row>
     <row r="41" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B41" s="2">
-        <v>6</v>
+        <v>1.5</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>110</v>
@@ -3351,16 +3404,16 @@
         <v>117</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G41" s="2">
-        <v>24.934650000000001</v>
+        <v>25.215733329999999</v>
       </c>
       <c r="H41" s="2">
-        <v>-80.548766670000006</v>
+        <v>-80.228566670000006</v>
       </c>
       <c r="I41" s="2">
         <v>100</v>
@@ -3374,10 +3427,10 @@
     </row>
     <row r="42" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B42" s="2">
-        <v>19</v>
+        <v>1.5</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>110</v>
@@ -3386,16 +3439,16 @@
         <v>117</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G42" s="2">
-        <v>24.934650000000001</v>
+        <v>25.215733329999999</v>
       </c>
       <c r="H42" s="2">
-        <v>-80.548766670000006</v>
+        <v>-80.228566670000006</v>
       </c>
       <c r="I42" s="2">
         <v>100</v>
@@ -3409,10 +3462,10 @@
     </row>
     <row r="43" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B43" s="2">
-        <v>1</v>
+        <v>8.5</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>110</v>
@@ -3421,16 +3474,16 @@
         <v>117</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G43" s="2">
-        <v>24.934650000000001</v>
+        <v>25.215733329999999</v>
       </c>
       <c r="H43" s="2">
-        <v>-80.548766670000006</v>
+        <v>-80.228566670000006</v>
       </c>
       <c r="I43" s="2">
         <v>100</v>
@@ -3444,10 +3497,10 @@
     </row>
     <row r="44" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="B44" s="2">
-        <v>3.5</v>
+        <v>22.5</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>110</v>
@@ -3456,16 +3509,16 @@
         <v>117</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G44" s="2">
-        <v>24.934650000000001</v>
+        <v>25.215733329999999</v>
       </c>
       <c r="H44" s="2">
-        <v>-80.548766670000006</v>
+        <v>-80.228566670000006</v>
       </c>
       <c r="I44" s="2">
         <v>100</v>
@@ -3479,10 +3532,10 @@
     </row>
     <row r="45" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B45" s="2">
-        <v>6</v>
+        <v>129</v>
+      </c>
+      <c r="B45" s="10">
+        <v>4</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>110</v>
@@ -3491,16 +3544,16 @@
         <v>117</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="G45" s="2">
-        <v>24.934650000000001</v>
+        <v>25.215733329999999</v>
       </c>
       <c r="H45" s="2">
-        <v>-80.548766670000006</v>
+        <v>-80.228566670000006</v>
       </c>
       <c r="I45" s="2">
         <v>100</v>
@@ -3514,10 +3567,10 @@
     </row>
     <row r="46" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>126</v>
+        <v>32</v>
       </c>
       <c r="B46" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>110</v>
@@ -3549,30 +3602,30 @@
     </row>
     <row r="47" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B47">
-        <v>7.5</v>
+        <v>82</v>
+      </c>
+      <c r="B47" s="2">
+        <v>6</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E47" t="s">
-        <v>122</v>
-      </c>
-      <c r="F47" t="s">
-        <v>123</v>
-      </c>
-      <c r="G47">
-        <v>24.521383329999999</v>
-      </c>
-      <c r="H47">
-        <v>-81.700149999999994</v>
-      </c>
-      <c r="I47">
+      <c r="E47" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G47" s="2">
+        <v>24.934650000000001</v>
+      </c>
+      <c r="H47" s="2">
+        <v>-80.548766670000006</v>
+      </c>
+      <c r="I47" s="2">
         <v>100</v>
       </c>
       <c r="J47" s="8" t="s">
@@ -3584,30 +3637,30 @@
     </row>
     <row r="48" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="B48">
-        <v>14.5</v>
+        <v>66</v>
+      </c>
+      <c r="B48" s="2">
+        <v>19</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E48" t="s">
-        <v>122</v>
-      </c>
-      <c r="F48" t="s">
-        <v>123</v>
-      </c>
-      <c r="G48">
-        <v>24.521383329999999</v>
-      </c>
-      <c r="H48">
-        <v>-81.700149999999994</v>
-      </c>
-      <c r="I48">
+      <c r="E48" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G48" s="2">
+        <v>24.934650000000001</v>
+      </c>
+      <c r="H48" s="2">
+        <v>-80.548766670000006</v>
+      </c>
+      <c r="I48" s="2">
         <v>100</v>
       </c>
       <c r="J48" s="8" t="s">
@@ -3619,30 +3672,30 @@
     </row>
     <row r="49" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B49">
-        <v>4</v>
+        <v>27</v>
+      </c>
+      <c r="B49" s="2">
+        <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E49" t="s">
-        <v>122</v>
-      </c>
-      <c r="F49" t="s">
-        <v>123</v>
-      </c>
-      <c r="G49">
-        <v>24.521383329999999</v>
-      </c>
-      <c r="H49">
-        <v>-81.700149999999994</v>
-      </c>
-      <c r="I49">
+      <c r="E49" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G49" s="2">
+        <v>24.934650000000001</v>
+      </c>
+      <c r="H49" s="2">
+        <v>-80.548766670000006</v>
+      </c>
+      <c r="I49" s="2">
         <v>100</v>
       </c>
       <c r="J49" s="8" t="s">
@@ -3654,30 +3707,30 @@
     </row>
     <row r="50" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B50">
-        <v>1.5</v>
+        <v>59</v>
+      </c>
+      <c r="B50" s="2">
+        <v>3.5</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E50" t="s">
-        <v>122</v>
-      </c>
-      <c r="F50" t="s">
-        <v>123</v>
-      </c>
-      <c r="G50">
-        <v>24.521383329999999</v>
-      </c>
-      <c r="H50">
-        <v>-81.700149999999994</v>
-      </c>
-      <c r="I50">
+      <c r="E50" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G50" s="2">
+        <v>24.934650000000001</v>
+      </c>
+      <c r="H50" s="2">
+        <v>-80.548766670000006</v>
+      </c>
+      <c r="I50" s="2">
         <v>100</v>
       </c>
       <c r="J50" s="8" t="s">
@@ -3689,30 +3742,30 @@
     </row>
     <row r="51" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B51">
-        <v>1</v>
+        <v>28</v>
+      </c>
+      <c r="B51" s="2">
+        <v>6</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E51" t="s">
-        <v>122</v>
-      </c>
-      <c r="F51" t="s">
-        <v>123</v>
-      </c>
-      <c r="G51">
-        <v>24.521383329999999</v>
-      </c>
-      <c r="H51">
-        <v>-81.700149999999994</v>
-      </c>
-      <c r="I51">
+      <c r="E51" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G51" s="2">
+        <v>24.934650000000001</v>
+      </c>
+      <c r="H51" s="2">
+        <v>-80.548766670000006</v>
+      </c>
+      <c r="I51" s="2">
         <v>100</v>
       </c>
       <c r="J51" s="8" t="s">
@@ -3724,30 +3777,30 @@
     </row>
     <row r="52" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52">
-        <v>4.5</v>
+        <v>126</v>
+      </c>
+      <c r="B52" s="2">
+        <v>2</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E52" t="s">
-        <v>122</v>
-      </c>
-      <c r="F52" t="s">
-        <v>123</v>
-      </c>
-      <c r="G52">
-        <v>24.521383329999999</v>
-      </c>
-      <c r="H52">
-        <v>-81.700149999999994</v>
-      </c>
-      <c r="I52">
+      <c r="E52" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G52" s="2">
+        <v>24.934650000000001</v>
+      </c>
+      <c r="H52" s="2">
+        <v>-80.548766670000006</v>
+      </c>
+      <c r="I52" s="2">
         <v>100</v>
       </c>
       <c r="J52" s="8" t="s">
@@ -3759,10 +3812,10 @@
     </row>
     <row r="53" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="B53">
-        <v>4.5</v>
+        <v>7.5</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>31</v>
@@ -3794,10 +3847,10 @@
     </row>
     <row r="54" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="B54">
-        <v>8</v>
+        <v>14.5</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>31</v>
@@ -3829,10 +3882,10 @@
     </row>
     <row r="55" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="B55">
-        <v>19.5</v>
+        <v>4</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>31</v>
@@ -3864,10 +3917,10 @@
     </row>
     <row r="56" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B56">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>31</v>
@@ -3876,16 +3929,16 @@
         <v>117</v>
       </c>
       <c r="E56" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F56" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G56">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H56">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I56">
         <v>100</v>
@@ -3899,10 +3952,10 @@
     </row>
     <row r="57" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="B57">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>31</v>
@@ -3911,16 +3964,16 @@
         <v>117</v>
       </c>
       <c r="E57" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F57" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G57">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H57">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I57">
         <v>100</v>
@@ -3934,10 +3987,10 @@
     </row>
     <row r="58" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>31</v>
@@ -3946,16 +3999,16 @@
         <v>117</v>
       </c>
       <c r="E58" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F58" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G58">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H58">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I58">
         <v>100</v>
@@ -3969,10 +4022,10 @@
     </row>
     <row r="59" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B59">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>31</v>
@@ -3981,16 +4034,16 @@
         <v>117</v>
       </c>
       <c r="E59" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F59" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G59">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H59">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I59">
         <v>100</v>
@@ -4004,10 +4057,10 @@
     </row>
     <row r="60" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B60">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>31</v>
@@ -4016,16 +4069,16 @@
         <v>117</v>
       </c>
       <c r="E60" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F60" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G60">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H60">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I60">
         <v>100</v>
@@ -4039,10 +4092,10 @@
     </row>
     <row r="61" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>59</v>
+        <v>126</v>
       </c>
       <c r="B61">
-        <v>6.5</v>
+        <v>19.5</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>31</v>
@@ -4051,16 +4104,16 @@
         <v>117</v>
       </c>
       <c r="E61" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F61" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G61">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H61">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I61">
         <v>100</v>
@@ -4074,10 +4127,10 @@
     </row>
     <row r="62" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="B62">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>31</v>
@@ -4086,16 +4139,16 @@
         <v>117</v>
       </c>
       <c r="E62" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F62" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="G62">
-        <v>24.4832</v>
+        <v>24.521383329999999</v>
       </c>
       <c r="H62">
-        <v>-81.946716670000001</v>
+        <v>-81.700149999999994</v>
       </c>
       <c r="I62">
         <v>100</v>
@@ -4109,10 +4162,10 @@
     </row>
     <row r="63" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>4.5</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>31</v>
@@ -4144,10 +4197,10 @@
     </row>
     <row r="64" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>126</v>
+        <v>73</v>
       </c>
       <c r="B64">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>31</v>
@@ -4177,82 +4230,322 @@
         <v>128</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-    </row>
-    <row r="66" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-    </row>
-    <row r="67" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-    </row>
-    <row r="68" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-    </row>
-    <row r="69" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-    </row>
-    <row r="70" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-    </row>
-    <row r="71" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-    </row>
-    <row r="72" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A72" s="2"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-    </row>
-    <row r="73" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A65" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E65" t="s">
+        <v>124</v>
+      </c>
+      <c r="F65" t="s">
+        <v>125</v>
+      </c>
+      <c r="G65">
+        <v>24.4832</v>
+      </c>
+      <c r="H65">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I65">
+        <v>100</v>
+      </c>
+      <c r="J65" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K65" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A66" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B66">
+        <v>3</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E66" t="s">
+        <v>124</v>
+      </c>
+      <c r="F66" t="s">
+        <v>125</v>
+      </c>
+      <c r="G66">
+        <v>24.4832</v>
+      </c>
+      <c r="H66">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I66">
+        <v>100</v>
+      </c>
+      <c r="J66" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K66" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A67" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B67">
+        <v>1.5</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E67" t="s">
+        <v>124</v>
+      </c>
+      <c r="F67" t="s">
+        <v>125</v>
+      </c>
+      <c r="G67">
+        <v>24.4832</v>
+      </c>
+      <c r="H67">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I67">
+        <v>100</v>
+      </c>
+      <c r="J67" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K67" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A68" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B68">
+        <v>6.5</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E68" t="s">
+        <v>124</v>
+      </c>
+      <c r="F68" t="s">
+        <v>125</v>
+      </c>
+      <c r="G68">
+        <v>24.4832</v>
+      </c>
+      <c r="H68">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I68">
+        <v>100</v>
+      </c>
+      <c r="J68" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K68" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A69" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B69">
+        <v>3</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E69" t="s">
+        <v>124</v>
+      </c>
+      <c r="F69" t="s">
+        <v>125</v>
+      </c>
+      <c r="G69">
+        <v>24.4832</v>
+      </c>
+      <c r="H69">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I69">
+        <v>100</v>
+      </c>
+      <c r="J69" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K69" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A70" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E70" t="s">
+        <v>124</v>
+      </c>
+      <c r="F70" t="s">
+        <v>125</v>
+      </c>
+      <c r="G70">
+        <v>24.4832</v>
+      </c>
+      <c r="H70">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I70">
+        <v>100</v>
+      </c>
+      <c r="J70" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K70" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A71" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B71">
+        <v>18</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E71" t="s">
+        <v>124</v>
+      </c>
+      <c r="F71" t="s">
+        <v>125</v>
+      </c>
+      <c r="G71">
+        <v>24.4832</v>
+      </c>
+      <c r="H71">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I71">
+        <v>100</v>
+      </c>
+      <c r="J71" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K71" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A72" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B72">
+        <v>4</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E72" t="s">
+        <v>124</v>
+      </c>
+      <c r="F72" t="s">
+        <v>132</v>
+      </c>
+      <c r="G72">
+        <v>24.4832</v>
+      </c>
+      <c r="H72">
+        <v>-81.946716670000001</v>
+      </c>
+      <c r="I72">
+        <v>100</v>
+      </c>
+      <c r="J72" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K72" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
     </row>
-    <row r="74" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
     </row>
-    <row r="75" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="2"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
     </row>
-    <row r="76" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
     </row>
-    <row r="77" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
     </row>
-    <row r="78" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
     </row>
-    <row r="79" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
     </row>
-    <row r="80" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -8787,42 +9080,42 @@
       <c r="C986" s="2"/>
       <c r="D986" s="2"/>
     </row>
-    <row r="987" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="987" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A987" s="2"/>
       <c r="C987" s="2"/>
       <c r="D987" s="2"/>
     </row>
-    <row r="988" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="988" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A988" s="2"/>
       <c r="C988" s="2"/>
       <c r="D988" s="2"/>
     </row>
-    <row r="989" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="989" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A989" s="2"/>
       <c r="C989" s="2"/>
       <c r="D989" s="2"/>
     </row>
-    <row r="990" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="990" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A990" s="2"/>
       <c r="C990" s="2"/>
       <c r="D990" s="2"/>
     </row>
-    <row r="991" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="991" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A991" s="2"/>
       <c r="C991" s="2"/>
       <c r="D991" s="2"/>
     </row>
-    <row r="992" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="992" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A992" s="2"/>
       <c r="C992" s="2"/>
       <c r="D992" s="2"/>
     </row>
-    <row r="993" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="993" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A993" s="2"/>
       <c r="C993" s="2"/>
       <c r="D993" s="2"/>
     </row>
-    <row r="994" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="994" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A994" s="2"/>
       <c r="C994" s="2"/>
       <c r="D994" s="2"/>
@@ -8857,15 +9150,56 @@
       <c r="C1000" s="2"/>
       <c r="D1000" s="2"/>
     </row>
+    <row r="1001" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1001" s="2"/>
+      <c r="C1001" s="2"/>
+      <c r="D1001" s="2"/>
+    </row>
+    <row r="1002" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1002" s="2"/>
+      <c r="C1002" s="2"/>
+      <c r="D1002" s="2"/>
+    </row>
+    <row r="1003" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1003" s="2"/>
+      <c r="C1003" s="2"/>
+      <c r="D1003" s="2"/>
+    </row>
+    <row r="1004" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1004" s="2"/>
+      <c r="C1004" s="2"/>
+      <c r="D1004" s="2"/>
+    </row>
+    <row r="1005" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1005" s="2"/>
+      <c r="C1005" s="2"/>
+      <c r="D1005" s="2"/>
+    </row>
+    <row r="1006" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1006" s="2"/>
+      <c r="C1006" s="2"/>
+      <c r="D1006" s="2"/>
+    </row>
+    <row r="1007" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1007" s="2"/>
+      <c r="C1007" s="2"/>
+      <c r="D1007" s="2"/>
+    </row>
+    <row r="1008" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1008" s="2"/>
+      <c r="C1008" s="2"/>
+      <c r="D1008" s="2"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D8 D47:D1000" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D53:D1008 D2:D10" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"Inshore,MidChannel,Offshore,Bank,Lagoon,ForeReef"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D9:D46" xr:uid="{CBFD8598-9A7D-4838-8036-0899C5C3EABA}">
-      <formula1>IF(C9="DryTortugas",        RangeDRTO,    IF(ISNUMBER(MATCH(C9, SubregionList, 0)),        RangeA,     SEFCRI))</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D11:D52" xr:uid="{CBFD8598-9A7D-4838-8036-0899C5C3EABA}">
+      <formula1>IF(C11="DryTortugas",        RangeDRTO,    IF(ISNUMBER(MATCH(C11, SubregionList, 0)),        RangeA,     SEFCRI))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1000" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1008" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"DryTortugas,LowerKeys,MiddleKeys,UpperKeys,Biscayne,SoutheastFlorida"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8876,9 +9210,9 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
-            <xm:f>Taxa!$A$2:$A$76</xm:f>
+            <xm:f>Taxa!$A$2:$A$77</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A8 A47:A1000</xm:sqref>
+          <xm:sqref>A2:A1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -8888,7 +9222,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:A996"/>
+  <dimension ref="A1:A997"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="26" width="8.59765625" customWidth="1"/>
@@ -8905,376 +9239,380 @@
       </c>
     </row>
     <row r="3" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
+      <c r="A3" s="9" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="6" t="s">
+    <row r="37" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="6" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="51" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>86</v>
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="58" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="59" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="62" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="63" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
-        <v>59</v>
+        <v>98</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="72" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A75" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="75" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" s="7" t="s">
+    <row r="76" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A76" s="7" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="76" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A76" s="2" t="s">
+    <row r="77" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A77" s="2" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="77" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="78" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="79" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="80" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -10194,6 +10532,7 @@
     <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -10202,6 +10541,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
@@ -10210,15 +10558,6 @@
     <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10417,20 +10756,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A51B496-5B66-49CD-B810-EE45484F45CB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{912B1377-D028-4F6B-BCA3-FAA07CA913FB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
     <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A51B496-5B66-49CD-B810-EE45484F45CB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>